<commit_message>
QA final: 14 correcciones (cierre con distancias parciales, fechas locales, botón atrás, deshacer, teclado), APK v1.0.0 y README
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011KyzW78AzQcMLMrpuMAmJW
</commit_message>
<xml_diff>
--- a/docs/ejemplos/proyecto.xlsx
+++ b/docs/ejemplos/proyecto.xlsx
@@ -3104,10 +3104,10 @@
         <v>VAd (−)</v>
       </c>
       <c r="F12" t="str">
-        <v>Dist. adelante/VI (m)</v>
+        <v>Dist. VAd/VI (VA en el BM inicial) (m)</v>
       </c>
       <c r="G12" t="str">
-        <v>Dist. atrás PC (m)</v>
+        <v>Dist. VA en PC (m)</v>
       </c>
       <c r="H12" t="str">
         <v>Subida</v>
@@ -3815,10 +3815,10 @@
         <v>VAd (−)</v>
       </c>
       <c r="F12" t="str">
-        <v>Dist. adelante/VI (m)</v>
+        <v>Dist. VAd/VI (VA en el BM inicial) (m)</v>
       </c>
       <c r="G12" t="str">
-        <v>Dist. atrás PC (m)</v>
+        <v>Dist. VA en PC (m)</v>
       </c>
       <c r="H12" t="str">
         <v>Subida</v>

</xml_diff>